<commit_message>
initial the report writing logic
</commit_message>
<xml_diff>
--- a/src/main/resources/files/report.xlsx
+++ b/src/main/resources/files/report.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2A8D3FA9-AC12-4124-984E-36A10B86F87E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{2AC6C071-75F1-439C-A90F-D47599B7CABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -12,7 +12,7 @@
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+    <ext uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="47">
   <si>
     <t>DATE</t>
   </si>
@@ -120,6 +120,75 @@
   </si>
   <si>
     <t xml:space="preserve">TOTAL </t>
+  </si>
+  <si>
+    <t>010831</t>
+  </si>
+  <si>
+    <t>31/08 - 12/09/2026</t>
+  </si>
+  <si>
+    <t>987654321RT0002</t>
+  </si>
+  <si>
+    <t>Sarah Jenkins</t>
+  </si>
+  <si>
+    <t>4200 University Ave, Unit 12</t>
+  </si>
+  <si>
+    <t>Mississauga, ON L5L 1C6</t>
+  </si>
+  <si>
+    <t>The site(s): 100 King Street West, Toronto, ON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	333 Bay Street, Toronto, ON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	31/08 - 05/09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	07/09 - 12/09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hours 		</t>
+  </si>
+  <si>
+    <t>40.0</t>
+  </si>
+  <si>
+    <t>37.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">My hours 		</t>
+  </si>
+  <si>
+    <t>77.50</t>
+  </si>
+  <si>
+    <t>82.0</t>
+  </si>
+  <si>
+    <t>3280</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>3075</t>
+  </si>
+  <si>
+    <t>6355</t>
+  </si>
+  <si>
+    <t>826</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>7181</t>
   </si>
 </sst>
 </file>
@@ -129,7 +198,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,12 +300,6 @@
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="3" tint="-0.249977111117893"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -255,6 +318,19 @@
       <b/>
       <sz val="13"/>
       <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF13284B"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3" tint="-0.249977111117893"/>
       <name val="Arial"/>
     </font>
   </fonts>
@@ -278,7 +354,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -367,17 +443,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF2B4C7E"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF2B4C7E"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color rgb="FF000000"/>
@@ -494,32 +559,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF2B4C7E"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF2B4C7E"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF2B4C7E"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF2B4C7E"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="dashed">
         <color rgb="FF000000"/>
       </left>
@@ -633,21 +672,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF2B4C7E"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF2B4C7E"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF2B4C7E"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="dashed">
         <color rgb="FF000000"/>
       </left>
@@ -692,6 +716,162 @@
       <top/>
       <bottom style="thin">
         <color rgb="FF2B4C7E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF2B4C7E"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF2B4C7E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF2B4C7E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="dashed">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF2B4C7E"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF2B4C7E"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF2B4C7E"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF2B4C7E"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF2B4C7E"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -699,7 +879,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="104">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -715,22 +895,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -745,77 +924,83 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="3" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
@@ -823,52 +1008,40 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -884,40 +1057,40 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -929,18 +1102,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -948,24 +1116,58 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1273,481 +1475,553 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:Q28"/>
+  <dimension ref="B2:Q29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="3" max="3" width="5.85546875" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" customWidth="1"/>
-    <col min="6" max="6" width="8.7109375" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" customWidth="1"/>
-    <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="10" max="10" width="11.5703125" customWidth="1"/>
-    <col min="11" max="11" width="6.85546875" customWidth="1"/>
-    <col min="12" max="12" width="7.7109375" customWidth="1"/>
-    <col min="13" max="13" width="9.85546875" customWidth="1"/>
-    <col min="14" max="14" width="5.42578125" customWidth="1"/>
+    <col min="3" max="3" customWidth="true" width="5.85546875"/>
+    <col min="4" max="4" customWidth="true" width="6.7109375"/>
+    <col min="5" max="5" customWidth="true" width="10.85546875"/>
+    <col min="6" max="6" customWidth="true" width="8.7109375"/>
+    <col min="7" max="7" customWidth="true" width="12.0"/>
+    <col min="8" max="8" customWidth="true" width="12.85546875"/>
+    <col min="9" max="9" customWidth="true" width="12.0"/>
+    <col min="10" max="10" customWidth="true" width="9.5703125"/>
+    <col min="11" max="11" customWidth="true" width="4.85546875"/>
+    <col min="12" max="12" customWidth="true" width="7.7109375"/>
+    <col min="13" max="13" customWidth="true" width="9.85546875"/>
+    <col min="14" max="14" customWidth="true" width="5.42578125"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:17">
       <c r="F2" s="3"/>
     </row>
     <row r="3" spans="2:17" ht="24.75" customHeight="1">
-      <c r="C3" s="11"/>
-      <c r="D3" s="43"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="44"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
-      <c r="J3" s="81"/>
-      <c r="K3" s="81"/>
-      <c r="L3" s="81"/>
-      <c r="M3" s="90"/>
-      <c r="N3" s="90"/>
-      <c r="O3" s="8"/>
+      <c r="J3" s="78"/>
+      <c r="K3" s="78"/>
+      <c r="L3" s="78"/>
+      <c r="M3" s="84" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="84"/>
+      <c r="O3" s="7"/>
     </row>
     <row r="4" spans="2:17" ht="19.5" customHeight="1">
-      <c r="C4" s="11"/>
-      <c r="D4" s="43"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="44"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
-      <c r="J4" s="32" t="s">
+      <c r="J4" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="K4" s="49"/>
-      <c r="L4" s="49"/>
-      <c r="M4" s="49"/>
-      <c r="N4" s="50"/>
-      <c r="O4" s="8"/>
+      <c r="K4" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="L4" s="47"/>
+      <c r="M4" s="47"/>
+      <c r="N4" s="48"/>
+      <c r="O4" s="7"/>
     </row>
     <row r="5" spans="2:17" ht="21.75" customHeight="1">
-      <c r="B5" s="13"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="43"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="44"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
-      <c r="J5" s="25" t="s">
+      <c r="J5" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="K5" s="49"/>
-      <c r="L5" s="49"/>
-      <c r="M5" s="49"/>
-      <c r="N5" s="50"/>
-      <c r="O5" s="8"/>
-      <c r="Q5" s="10"/>
+      <c r="K5" s="49" t="s">
+        <v>26</v>
+      </c>
+      <c r="L5" s="47"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="48"/>
+      <c r="O5" s="7"/>
+      <c r="Q5" s="9"/>
     </row>
     <row r="6" spans="2:17" ht="8.25" customHeight="1">
-      <c r="B6" s="13"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="12"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="82"/>
-      <c r="K6" s="82"/>
-      <c r="L6" s="82"/>
-      <c r="M6" s="82"/>
-      <c r="N6" s="82"/>
-      <c r="O6" s="8"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="10"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="79"/>
+      <c r="K6" s="79"/>
+      <c r="L6" s="79"/>
+      <c r="M6" s="79"/>
+      <c r="N6" s="79"/>
+      <c r="O6" s="7"/>
     </row>
     <row r="7" spans="2:17" ht="21.75" customHeight="1">
-      <c r="B7" s="13"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="23" t="s">
+      <c r="B7" s="12"/>
+      <c r="C7" s="10"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="F7" s="51" t="s">
+      <c r="F7" s="50" t="s">
         <v>3</v>
       </c>
-      <c r="G7" s="51"/>
-      <c r="H7" s="52"/>
-      <c r="I7" s="18" t="s">
+      <c r="G7" s="50"/>
+      <c r="H7" s="51"/>
+      <c r="I7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="J7" s="51"/>
-      <c r="K7" s="51"/>
-      <c r="L7" s="51"/>
-      <c r="M7" s="51"/>
-      <c r="N7" s="53"/>
-      <c r="O7" s="8"/>
+      <c r="J7" s="50" t="s">
+        <v>27</v>
+      </c>
+      <c r="K7" s="50"/>
+      <c r="L7" s="50"/>
+      <c r="M7" s="50"/>
+      <c r="N7" s="52"/>
+      <c r="O7" s="7"/>
     </row>
     <row r="8" spans="2:17" ht="21.75" customHeight="1">
-      <c r="B8" s="13"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="24" t="s">
+      <c r="B8" s="12"/>
+      <c r="C8" s="10"/>
+      <c r="D8" s="44"/>
+      <c r="E8" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="F8" s="51" t="s">
+      <c r="F8" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="G8" s="51"/>
-      <c r="H8" s="52"/>
-      <c r="I8" s="20" t="s">
+      <c r="G8" s="50"/>
+      <c r="H8" s="51"/>
+      <c r="I8" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="J8" s="51"/>
-      <c r="K8" s="51"/>
-      <c r="L8" s="51"/>
-      <c r="M8" s="51"/>
-      <c r="N8" s="53"/>
-      <c r="O8" s="8"/>
+      <c r="J8" s="50" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" s="50"/>
+      <c r="L8" s="50"/>
+      <c r="M8" s="50"/>
+      <c r="N8" s="52"/>
+      <c r="O8" s="7"/>
     </row>
     <row r="9" spans="2:17" ht="21" customHeight="1">
-      <c r="B9" s="13"/>
-      <c r="C9" s="11"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="51" t="s">
+      <c r="B9" s="12"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="44"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="G9" s="51"/>
-      <c r="H9" s="52"/>
-      <c r="I9" s="19"/>
-      <c r="J9" s="51"/>
-      <c r="K9" s="51"/>
-      <c r="L9" s="51"/>
-      <c r="M9" s="51"/>
-      <c r="N9" s="53"/>
-      <c r="O9" s="8"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="K9" s="50"/>
+      <c r="L9" s="50"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="52"/>
+      <c r="O9" s="7"/>
     </row>
     <row r="10" spans="2:17" ht="16.5" customHeight="1">
-      <c r="B10" s="13"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="59"/>
-      <c r="G10" s="59"/>
-      <c r="H10" s="60"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="51"/>
-      <c r="K10" s="51"/>
-      <c r="L10" s="51"/>
-      <c r="M10" s="51"/>
-      <c r="N10" s="53"/>
-      <c r="O10" s="8"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="56"/>
+      <c r="G10" s="56"/>
+      <c r="H10" s="57"/>
+      <c r="I10" s="45"/>
+      <c r="J10" s="50"/>
+      <c r="K10" s="50"/>
+      <c r="L10" s="50"/>
+      <c r="M10" s="50"/>
+      <c r="N10" s="52"/>
+      <c r="O10" s="7"/>
     </row>
     <row r="11" spans="2:17" ht="8.25" customHeight="1">
-      <c r="B11" s="13"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="43"/>
-      <c r="E11" s="81"/>
-      <c r="F11" s="81"/>
-      <c r="G11" s="81"/>
-      <c r="H11" s="81"/>
-      <c r="I11" s="81"/>
-      <c r="J11" s="81"/>
-      <c r="K11" s="81"/>
-      <c r="L11" s="81"/>
-      <c r="M11" s="81"/>
-      <c r="N11" s="81"/>
-      <c r="O11" s="8"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="44"/>
+      <c r="E11" s="78"/>
+      <c r="F11" s="78"/>
+      <c r="G11" s="78"/>
+      <c r="H11" s="78"/>
+      <c r="I11" s="78"/>
+      <c r="J11" s="78"/>
+      <c r="K11" s="78"/>
+      <c r="L11" s="78"/>
+      <c r="M11" s="78"/>
+      <c r="N11" s="78"/>
+      <c r="O11" s="7"/>
     </row>
     <row r="12" spans="2:17" ht="24" customHeight="1">
-      <c r="B12" s="13"/>
-      <c r="C12" s="78" t="s">
+      <c r="B12" s="12"/>
+      <c r="C12" s="75" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="79" t="s">
+      <c r="D12" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="E12" s="56" t="s">
+      <c r="E12" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="F12" s="57"/>
-      <c r="G12" s="56" t="s">
+      <c r="F12" s="54"/>
+      <c r="G12" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="H12" s="58"/>
-      <c r="I12" s="96" t="s">
+      <c r="H12" s="55"/>
+      <c r="I12" s="85" t="s">
         <v>12</v>
       </c>
-      <c r="J12" s="96"/>
-      <c r="K12" s="96" t="s">
+      <c r="J12" s="85"/>
+      <c r="K12" s="85" t="s">
         <v>13</v>
       </c>
-      <c r="L12" s="96"/>
-      <c r="M12" s="96" t="s">
+      <c r="L12" s="85"/>
+      <c r="M12" s="85" t="s">
         <v>14</v>
       </c>
-      <c r="N12" s="97"/>
-      <c r="O12" s="8"/>
+      <c r="N12" s="86"/>
+      <c r="O12" s="7"/>
     </row>
     <row r="13" spans="2:17" ht="8.25" customHeight="1">
-      <c r="B13" s="13"/>
-      <c r="C13" s="78"/>
-      <c r="D13" s="80"/>
-      <c r="E13" s="85"/>
-      <c r="F13" s="86"/>
-      <c r="G13" s="86"/>
-      <c r="H13" s="86"/>
-      <c r="I13" s="89"/>
-      <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="91"/>
-      <c r="N13" s="91"/>
-      <c r="O13" s="8"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="75"/>
+      <c r="D13" s="77"/>
+      <c r="E13" s="80"/>
+      <c r="F13" s="80"/>
+      <c r="G13" s="80"/>
+      <c r="H13" s="80"/>
+      <c r="I13" s="83"/>
+      <c r="J13" s="87"/>
+      <c r="K13" s="87"/>
+      <c r="L13" s="87"/>
+      <c r="M13" s="83"/>
+      <c r="N13" s="83"/>
+      <c r="O13" s="7"/>
     </row>
     <row r="14" spans="2:17" ht="28.5" customHeight="1">
-      <c r="B14" s="13"/>
-      <c r="C14" s="78"/>
-      <c r="D14" s="80"/>
-      <c r="E14" s="31" t="s">
+      <c r="B14" s="12"/>
+      <c r="C14" s="75"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="103" t="s">
         <v>15</v>
       </c>
-      <c r="F14" s="94" t="s">
+      <c r="F14" s="98" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="95"/>
-      <c r="H14" s="95"/>
-      <c r="I14" s="95"/>
-      <c r="J14" s="54" t="s">
+      <c r="G14" s="97"/>
+      <c r="H14" s="97"/>
+      <c r="I14" s="99"/>
+      <c r="J14" s="100" t="s">
         <v>17</v>
       </c>
-      <c r="K14" s="55"/>
-      <c r="L14" s="45" t="s">
+      <c r="K14" s="101"/>
+      <c r="L14" s="102" t="s">
         <v>18</v>
       </c>
-      <c r="M14" s="83" t="s">
+      <c r="M14" s="96" t="s">
         <v>19</v>
       </c>
-      <c r="N14" s="84"/>
-      <c r="O14" s="8"/>
+      <c r="N14" s="97"/>
+      <c r="O14" s="7"/>
     </row>
     <row r="15" spans="2:17" ht="18" customHeight="1">
-      <c r="B15" s="13"/>
-      <c r="C15" s="78"/>
-      <c r="D15" s="80"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="92" t="s">
+      <c r="B15" s="12"/>
+      <c r="C15" s="75"/>
+      <c r="D15" s="77"/>
+      <c r="E15" s="92"/>
+      <c r="F15" s="88" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="93"/>
-      <c r="H15" s="93"/>
-      <c r="I15" s="93"/>
-      <c r="J15" s="33"/>
-      <c r="K15" s="26"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="37"/>
-      <c r="N15" s="38"/>
-      <c r="O15" s="8"/>
+      <c r="G15" s="89"/>
+      <c r="H15" s="89"/>
+      <c r="I15" s="89"/>
+      <c r="J15" s="90"/>
+      <c r="K15" s="91"/>
+      <c r="L15" s="93"/>
+      <c r="M15" s="94"/>
+      <c r="N15" s="95"/>
+      <c r="O15" s="7"/>
     </row>
     <row r="16" spans="2:17" ht="18" customHeight="1">
-      <c r="B16" s="13"/>
-      <c r="C16" s="78"/>
-      <c r="D16" s="80"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="87"/>
-      <c r="G16" s="88"/>
-      <c r="H16" s="88"/>
-      <c r="I16" s="88"/>
-      <c r="J16" s="33"/>
-      <c r="K16" s="26"/>
-      <c r="L16" s="27"/>
-      <c r="M16" s="37"/>
-      <c r="N16" s="38"/>
-      <c r="O16" s="8"/>
-    </row>
-    <row r="17" spans="2:16" ht="18" customHeight="1">
-      <c r="B17" s="13"/>
-      <c r="C17" s="78"/>
-      <c r="D17" s="80"/>
-      <c r="E17" s="17"/>
-      <c r="F17" s="63"/>
-      <c r="G17" s="64"/>
-      <c r="H17" s="64"/>
-      <c r="I17" s="64"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="26"/>
-      <c r="L17" s="27"/>
-      <c r="M17" s="37"/>
-      <c r="N17" s="38"/>
-      <c r="O17" s="8"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="75"/>
+      <c r="D16" s="77"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="81" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" s="82"/>
+      <c r="H16" s="82"/>
+      <c r="I16" s="82"/>
+      <c r="J16" s="31"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="26"/>
+      <c r="M16" s="35"/>
+      <c r="N16" s="36"/>
+      <c r="O16" s="7"/>
+    </row>
+    <row r="17" ht="18.0" customHeight="true">
+      <c r="E17" s="16"/>
+      <c r="F17" s="60" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="61"/>
+      <c r="H17" s="61"/>
+      <c r="I17" s="61"/>
+      <c r="J17" s="31"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="35"/>
+      <c r="N17" s="36"/>
     </row>
     <row r="18" spans="2:16" ht="18" customHeight="1">
-      <c r="B18" s="13"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="43"/>
-      <c r="E18" s="46"/>
-      <c r="F18" s="70"/>
-      <c r="G18" s="71"/>
-      <c r="H18" s="71"/>
-      <c r="I18" s="48"/>
-      <c r="J18" s="47"/>
-      <c r="K18" s="26"/>
-      <c r="L18" s="27"/>
-      <c r="M18" s="37"/>
-      <c r="N18" s="38"/>
-      <c r="O18" s="8"/>
-      <c r="P18" s="3"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="75"/>
+      <c r="D18" s="77"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="60" t="s">
+        <v>32</v>
+      </c>
+      <c r="G18" s="61"/>
+      <c r="H18" s="61"/>
+      <c r="I18" s="61"/>
+      <c r="J18" s="31"/>
+      <c r="K18" s="25"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="35"/>
+      <c r="N18" s="36"/>
+      <c r="O18" s="7"/>
     </row>
     <row r="19" spans="2:16" ht="18" customHeight="1">
-      <c r="B19" s="13"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="66"/>
-      <c r="G19" s="67"/>
-      <c r="H19" s="67"/>
-      <c r="I19" s="67"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="26"/>
-      <c r="L19" s="27"/>
-      <c r="M19" s="37"/>
-      <c r="N19" s="38"/>
-      <c r="O19" s="8"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="44"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="67" t="s">
+        <v>34</v>
+      </c>
+      <c r="G19" s="68"/>
+      <c r="H19" s="68"/>
+      <c r="I19" s="43" t="s">
+        <v>35</v>
+      </c>
+      <c r="J19" s="42" t="s">
+        <v>39</v>
+      </c>
+      <c r="K19" s="25"/>
+      <c r="L19" s="26" t="s">
+        <v>35</v>
+      </c>
+      <c r="M19" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="N19" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="O19" s="7"/>
       <c r="P19" s="3"/>
     </row>
     <row r="20" spans="2:16" ht="18" customHeight="1">
-      <c r="B20" s="13"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="43"/>
-      <c r="E20" s="15"/>
-      <c r="F20" s="70"/>
-      <c r="G20" s="71"/>
-      <c r="H20" s="71"/>
-      <c r="I20" s="48"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="28"/>
-      <c r="L20" s="35"/>
-      <c r="M20" s="37"/>
-      <c r="N20" s="38"/>
-      <c r="O20" s="8"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="63" t="s">
+        <v>33</v>
+      </c>
+      <c r="G20" s="64"/>
+      <c r="H20" s="64"/>
+      <c r="I20" s="64"/>
+      <c r="J20" s="31"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="26"/>
+      <c r="M20" s="35"/>
+      <c r="N20" s="36"/>
+      <c r="O20" s="7"/>
       <c r="P20" s="3"/>
     </row>
     <row r="21" spans="2:16" ht="18" customHeight="1">
-      <c r="B21" s="13"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="70"/>
-      <c r="G21" s="71"/>
-      <c r="H21" s="71"/>
-      <c r="I21" s="48"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="26"/>
-      <c r="L21" s="27"/>
-      <c r="M21" s="37"/>
-      <c r="N21" s="38"/>
-      <c r="O21" s="8"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="10"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="67" t="s">
+        <v>34</v>
+      </c>
+      <c r="G21" s="68"/>
+      <c r="H21" s="68"/>
+      <c r="I21" s="43" t="s">
+        <v>36</v>
+      </c>
+      <c r="J21" s="32" t="s">
+        <v>39</v>
+      </c>
+      <c r="K21" s="27"/>
+      <c r="L21" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="M21" s="35" t="s">
+        <v>42</v>
+      </c>
+      <c r="N21" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="O21" s="7"/>
       <c r="P21" s="3"/>
     </row>
     <row r="22" spans="2:16" ht="18" customHeight="1">
-      <c r="B22" s="13"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="43"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="68"/>
-      <c r="G22" s="69"/>
-      <c r="H22" s="69"/>
-      <c r="I22" s="69"/>
-      <c r="J22" s="36"/>
-      <c r="K22" s="29"/>
-      <c r="L22" s="30"/>
-      <c r="M22" s="37"/>
-      <c r="N22" s="38"/>
-      <c r="O22" s="8"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="10"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="67" t="s">
+        <v>37</v>
+      </c>
+      <c r="G22" s="68"/>
+      <c r="H22" s="68"/>
+      <c r="I22" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="J22" s="33"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="26"/>
+      <c r="M22" s="35"/>
+      <c r="N22" s="36"/>
+      <c r="O22" s="7"/>
       <c r="P22" s="3"/>
     </row>
     <row r="23" spans="2:16" ht="18" customHeight="1">
-      <c r="B23" s="13"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="43"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="76" t="s">
+      <c r="B23" s="12"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="44"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="65"/>
+      <c r="G23" s="66"/>
+      <c r="H23" s="66"/>
+      <c r="I23" s="66"/>
+      <c r="J23" s="34"/>
+      <c r="K23" s="28"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="35" t="s">
+        <v>43</v>
+      </c>
+      <c r="N23" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="O23" s="7"/>
+      <c r="P23" s="3"/>
+    </row>
+    <row r="24" spans="2:16" ht="18" customHeight="1">
+      <c r="B24" s="12"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="5"/>
+      <c r="F24" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="G23" s="77"/>
-      <c r="H23" s="77"/>
-      <c r="I23" s="77"/>
-      <c r="J23" s="77"/>
-      <c r="K23" s="77"/>
-      <c r="L23" s="77"/>
-      <c r="M23" s="39"/>
-      <c r="N23" s="40"/>
-      <c r="O23" s="8"/>
-      <c r="P23" s="3"/>
-    </row>
-    <row r="24" spans="2:16" ht="18" customHeight="1">
-      <c r="B24" s="13"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="43"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="74" t="s">
+      <c r="G24" s="74"/>
+      <c r="H24" s="74"/>
+      <c r="I24" s="74"/>
+      <c r="J24" s="74"/>
+      <c r="K24" s="74"/>
+      <c r="L24" s="74"/>
+      <c r="M24" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="N24" s="38" t="s">
+        <v>45</v>
+      </c>
+      <c r="O24" s="7"/>
+      <c r="P24" s="3"/>
+    </row>
+    <row r="25" spans="2:16" ht="18" customHeight="1">
+      <c r="B25" s="12"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="44"/>
+      <c r="E25" s="5"/>
+      <c r="F25" s="71" t="s">
         <v>22</v>
       </c>
-      <c r="G24" s="75"/>
-      <c r="H24" s="75"/>
-      <c r="I24" s="75"/>
-      <c r="J24" s="75"/>
-      <c r="K24" s="75"/>
-      <c r="L24" s="75"/>
-      <c r="M24" s="39"/>
-      <c r="N24" s="40"/>
-      <c r="O24" s="8"/>
-      <c r="P24" s="3"/>
-    </row>
-    <row r="25" spans="2:16" ht="18" customHeight="1">
-      <c r="B25" s="13"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="43"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="72" t="s">
+      <c r="G25" s="72"/>
+      <c r="H25" s="72"/>
+      <c r="I25" s="72"/>
+      <c r="J25" s="72"/>
+      <c r="K25" s="72"/>
+      <c r="L25" s="72"/>
+      <c r="M25" s="37"/>
+      <c r="N25" s="38"/>
+      <c r="O25" s="7"/>
+      <c r="P25" s="3"/>
+    </row>
+    <row r="26" spans="2:16" ht="18" customHeight="1">
+      <c r="B26" s="12"/>
+      <c r="C26" s="10"/>
+      <c r="D26" s="44"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="69" t="s">
         <v>23</v>
       </c>
-      <c r="G25" s="73"/>
-      <c r="H25" s="73"/>
-      <c r="I25" s="73"/>
-      <c r="J25" s="73"/>
-      <c r="K25" s="73"/>
-      <c r="L25" s="73"/>
-      <c r="M25" s="41"/>
-      <c r="N25" s="42"/>
-      <c r="O25" s="8"/>
-      <c r="P25" s="3"/>
-    </row>
-    <row r="26" spans="2:16" ht="15.95" customHeight="1">
-      <c r="B26" s="13"/>
-      <c r="D26" s="6"/>
-      <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-      <c r="G26" s="6"/>
-      <c r="H26" s="6"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-      <c r="K26" s="6"/>
-      <c r="L26" s="6"/>
-      <c r="M26" s="6"/>
-      <c r="N26" s="6"/>
-      <c r="O26" s="8"/>
+      <c r="G26" s="70"/>
+      <c r="H26" s="70"/>
+      <c r="I26" s="70"/>
+      <c r="J26" s="70"/>
+      <c r="K26" s="70"/>
+      <c r="L26" s="70"/>
+      <c r="M26" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="N26" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="O26" s="7"/>
       <c r="P26" s="3"/>
     </row>
     <row r="27" spans="2:16" ht="15.95" customHeight="1">
-      <c r="B27" s="13"/>
-      <c r="L27" s="1"/>
-      <c r="M27" s="65"/>
-      <c r="N27" s="62"/>
+      <c r="B27" s="12"/>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
+      <c r="J27" s="6"/>
+      <c r="K27" s="6"/>
+      <c r="L27" s="6"/>
+      <c r="M27" s="6"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="7"/>
       <c r="P27" s="3"/>
     </row>
-    <row r="28" spans="2:16" ht="18" customHeight="1">
-      <c r="L28" s="2"/>
-      <c r="M28" s="61"/>
-      <c r="N28" s="62"/>
+    <row r="28" spans="2:16" ht="15.95" customHeight="1">
+      <c r="B28" s="12"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="62"/>
+      <c r="N28" s="59"/>
+      <c r="P28" s="3"/>
+    </row>
+    <row r="29" spans="2:16" ht="18" customHeight="1">
+      <c r="L29" s="2"/>
+      <c r="M29" s="58"/>
+      <c r="N29" s="59"/>
     </row>
   </sheetData>
-  <mergeCells count="40">
+  <mergeCells count="52">
     <mergeCell ref="C12:C17"/>
     <mergeCell ref="D12:D17"/>
     <mergeCell ref="J3:L3"/>
@@ -1764,17 +2038,6 @@
     <mergeCell ref="M12:N12"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="K12:L12"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="M27:N27"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="F22:I22"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="F25:L25"/>
-    <mergeCell ref="F24:L24"/>
-    <mergeCell ref="F23:L23"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F21:H21"/>
     <mergeCell ref="J14:K14"/>
     <mergeCell ref="J9:N9"/>
     <mergeCell ref="J10:N10"/>
@@ -1788,6 +2051,18 @@
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="J7:N7"/>
     <mergeCell ref="J8:N8"/>
+    <mergeCell ref="M29:N29"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="F26:L26"/>
+    <mergeCell ref="F25:L25"/>
+    <mergeCell ref="F24:L24"/>
+    <mergeCell ref="F21:H21"/>
+    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="F17:I17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
added the amount column in DB and basic HTML+CSS
</commit_message>
<xml_diff>
--- a/src/main/resources/files/report.xlsx
+++ b/src/main/resources/files/report.xlsx
@@ -155,16 +155,16 @@
     <t xml:space="preserve">hours 		</t>
   </si>
   <si>
-    <t>40.0</t>
-  </si>
-  <si>
-    <t>37.5</t>
+    <t>40:00</t>
+  </si>
+  <si>
+    <t>37:30</t>
   </si>
   <si>
     <t xml:space="preserve">My hours 		</t>
   </si>
   <si>
-    <t>77.50</t>
+    <t>77:30</t>
   </si>
   <si>
     <t>82.0</t>

</xml_diff>